<commit_message>
Test case y SRTM
Cuarta version del test case y  segunda version del SRTM
</commit_message>
<xml_diff>
--- a/Docs/SRTM_Proyecto_CNC.xlsx
+++ b/Docs/SRTM_Proyecto_CNC.xlsx
@@ -5,18 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yepes\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yepes\Documents\EIA\Septimo semestre\Embebidos\Proyecto\Test_Case_Video_Evidencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{581314A1-DDAA-41C3-8A84-31A155C8AF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012D2A64-4C9A-4D45-A14C-CD1BE1AADECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SRTM" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="144">
   <si>
     <t>Software Requirements Traceability Matrix (SRTM) - Proyecto CNC</t>
   </si>
@@ -90,9 +89,6 @@
     <t>HIL / System</t>
   </si>
   <si>
-    <t>Por confirmar</t>
-  </si>
-  <si>
     <t>Completar Actual Results después de ejecutar la prueba.</t>
   </si>
   <si>
@@ -444,44 +440,35 @@
     <t>Test_Case_Video_Evidencia/TC-006.mp4</t>
   </si>
   <si>
-    <t>Test_Case_Video_Evidencia/TC-003-Funcionamiento.mp4
+    <t>Test_Case_Video_Evidencia/TC-013.jpg</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-005.mp4
 Test_Case_Video_Evidencia/TC-003-Mediciones.jpg</t>
   </si>
   <si>
-    <t>Test_Case_Video_Evidencia/TC-007-Control_manual.mp4
-Test_Case_Video_Evidencia/TC-007-Homing.mp4</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-008.jpg</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-009-Corriente.jpg
-Test_Case_Video_Evidencia/TC-009-stop.mp4</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-010-mensajes.jpg
-Test_Case_Video_Evidencia/TC-010-indicadores.mp4</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-011.jpg</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-012.jpg</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-013.jpg</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-014.mp4</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-015.jpg</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-016.mp4</t>
-  </si>
-  <si>
-    <t>Test_Case_Video_Evidencia/TC-017.jpg</t>
+    <t>Test_Case_Video_Evidencia/TC-007.mp4</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-010.jpg</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-008.mp4</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-009.mp4</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-010.mp4</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>Test_Case_Video_Evidencia/TC-005.mp4
+Test_Case_Video_Evidencia/TC-008.mp4
+Test_Case_Video_Evidencia/TC-009.mp4
+Test_Case_Video_Evidencia/TC-010.mp4</t>
   </si>
 </sst>
 </file>
@@ -816,193 +803,193 @@
         <v>17</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="78" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>24</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>18</v>
+        <v>142</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="78" customHeight="1">
       <c r="A5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>136</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>18</v>
+        <v>142</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="78" customHeight="1">
       <c r="A6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="78" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="78" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="78" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>59</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>17</v>
@@ -1011,330 +998,324 @@
         <v>137</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>18</v>
+        <v>142</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="78" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>66</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="78" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="F11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="78" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="78" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="F13" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="78" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="F14" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="78" customHeight="1">
       <c r="A15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="F15" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="78" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="F16" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>108</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="78" customHeight="1">
       <c r="A17" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2"/>
+      <c r="I17" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="78" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="F18" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="G18" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="78" customHeight="1">
       <c r="A19" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>